<commit_message>
Post-game chapter, Shadow sprite sources, and updated project docs
- Bump pokeemerald-expansion to the post-game commit (Nessa's welcome and
  the Private Jet, the Armored Mewtwo chapter, the Shadow content wave,
  the recut credits, and the rewritten README).
- Add the 13 pogokitten Shadow sprite sources imported this round.
- Spawn documentation: Celebi Island fishing, Shadow Vaporeon on Routes
  129/130, the Shin-Tokyo patrol pools, Armored Mewtwo, and a new sheet
  listing every Shadow species with finished art but no encounter.
- Handoff log brought current through the post-game rounds.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Wishes_of_Tomorrow_Pokemon_by_Area.xlsx
+++ b/Wishes_of_Tomorrow_Pokemon_by_Area.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pokemon by Area" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unobtainable Shadows" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pokemon by Area'!$A$1:$F$101</definedName>
@@ -109,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -168,6 +169,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -533,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F101"/>
+  <dimension ref="A1:F119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -3412,6 +3414,554 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" s="22" t="inlineStr">
+        <is>
+          <t>Celebi Island</t>
+        </is>
+      </c>
+      <c r="B102" s="22" t="inlineStr">
+        <is>
+          <t>Fishing (Old Rod)</t>
+        </is>
+      </c>
+      <c r="C102" s="22" t="inlineStr">
+        <is>
+          <t>Azurill (Shadow)</t>
+        </is>
+      </c>
+      <c r="D102" s="22" t="inlineStr">
+        <is>
+          <t>30-34</t>
+        </is>
+      </c>
+      <c r="E102" s="22" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F102" s="22" t="inlineStr">
+        <is>
+          <t>Common; all island wilds are Shadow</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="22" t="inlineStr">
+        <is>
+          <t>Celebi Island</t>
+        </is>
+      </c>
+      <c r="B103" s="22" t="inlineStr">
+        <is>
+          <t>Fishing (Good Rod)</t>
+        </is>
+      </c>
+      <c r="C103" s="22" t="inlineStr">
+        <is>
+          <t>Azurill (Shadow)</t>
+        </is>
+      </c>
+      <c r="D103" s="22" t="inlineStr">
+        <is>
+          <t>32-36</t>
+        </is>
+      </c>
+      <c r="E103" s="22" t="inlineStr">
+        <is>
+          <t>80%</t>
+        </is>
+      </c>
+      <c r="F103" s="22" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="22" t="inlineStr">
+        <is>
+          <t>Celebi Island</t>
+        </is>
+      </c>
+      <c r="B104" s="22" t="inlineStr">
+        <is>
+          <t>Fishing (Good Rod)</t>
+        </is>
+      </c>
+      <c r="C104" s="22" t="inlineStr">
+        <is>
+          <t>Blastoise (Shadow)</t>
+        </is>
+      </c>
+      <c r="D104" s="22" t="inlineStr">
+        <is>
+          <t>36-40</t>
+        </is>
+      </c>
+      <c r="E104" s="22" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="F104" s="22" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="22" t="inlineStr">
+        <is>
+          <t>Celebi Island</t>
+        </is>
+      </c>
+      <c r="B105" s="22" t="inlineStr">
+        <is>
+          <t>Fishing (Super Rod)</t>
+        </is>
+      </c>
+      <c r="C105" s="22" t="inlineStr">
+        <is>
+          <t>Blastoise (Shadow)</t>
+        </is>
+      </c>
+      <c r="D105" s="22" t="inlineStr">
+        <is>
+          <t>38-44</t>
+        </is>
+      </c>
+      <c r="E105" s="22" t="inlineStr">
+        <is>
+          <t>~60%</t>
+        </is>
+      </c>
+      <c r="F105" s="22" t="inlineStr">
+        <is>
+          <t>Rare catch of the island</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="22" t="inlineStr">
+        <is>
+          <t>Celebi Island</t>
+        </is>
+      </c>
+      <c r="B106" s="22" t="inlineStr">
+        <is>
+          <t>Fishing (Super Rod)</t>
+        </is>
+      </c>
+      <c r="C106" s="22" t="inlineStr">
+        <is>
+          <t>Azurill (Shadow)</t>
+        </is>
+      </c>
+      <c r="D106" s="22" t="inlineStr">
+        <is>
+          <t>36-40</t>
+        </is>
+      </c>
+      <c r="E106" s="22" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="F106" s="22" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="22" t="inlineStr">
+        <is>
+          <t>Route 129</t>
+        </is>
+      </c>
+      <c r="B107" s="22" t="inlineStr">
+        <is>
+          <t>Surfing</t>
+        </is>
+      </c>
+      <c r="C107" s="22" t="inlineStr">
+        <is>
+          <t>Vaporeon (Shadow)</t>
+        </is>
+      </c>
+      <c r="D107" s="22" t="inlineStr">
+        <is>
+          <t>34-38</t>
+        </is>
+      </c>
+      <c r="E107" s="22" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="F107" s="22" t="inlineStr">
+        <is>
+          <t>Medium-rare; all route wilds are Shadow</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="22" t="inlineStr">
+        <is>
+          <t>Route 130</t>
+        </is>
+      </c>
+      <c r="B108" s="22" t="inlineStr">
+        <is>
+          <t>Surfing</t>
+        </is>
+      </c>
+      <c r="C108" s="22" t="inlineStr">
+        <is>
+          <t>Vaporeon (Shadow)</t>
+        </is>
+      </c>
+      <c r="D108" s="22" t="inlineStr">
+        <is>
+          <t>34-38</t>
+        </is>
+      </c>
+      <c r="E108" s="22" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="F108" s="22" t="inlineStr">
+        <is>
+          <t>Medium-rare; Route 130 wilds now Shadow too</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="22" t="inlineStr">
+        <is>
+          <t>Route 130</t>
+        </is>
+      </c>
+      <c r="B109" s="22" t="inlineStr">
+        <is>
+          <t>Surfing</t>
+        </is>
+      </c>
+      <c r="C109" s="22" t="inlineStr">
+        <is>
+          <t>Squirtle/Lanturn/Piplup/Politoed (Shadow)</t>
+        </is>
+      </c>
+      <c r="D109" s="22" t="inlineStr">
+        <is>
+          <t>30-38</t>
+        </is>
+      </c>
+      <c r="E109" s="22" t="inlineStr">
+        <is>
+          <t>see 129</t>
+        </is>
+      </c>
+      <c r="F109" s="22" t="inlineStr">
+        <is>
+          <t>Mirrors Route 129 table</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="22" t="inlineStr">
+        <is>
+          <t>Route 130</t>
+        </is>
+      </c>
+      <c r="B110" s="22" t="inlineStr">
+        <is>
+          <t>Fishing (all rods)</t>
+        </is>
+      </c>
+      <c r="C110" s="22" t="inlineStr">
+        <is>
+          <t>Same as Route 129 (Shadow)</t>
+        </is>
+      </c>
+      <c r="D110" s="22" t="inlineStr">
+        <is>
+          <t>30-42</t>
+        </is>
+      </c>
+      <c r="E110" s="22" t="inlineStr"/>
+      <c r="F110" s="22" t="inlineStr">
+        <is>
+          <t>Kingdra/Dragonair/Empoleon on Super Rod</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="22" t="inlineStr">
+        <is>
+          <t>Shin-Tokyo (Red Alert)</t>
+        </is>
+      </c>
+      <c r="B111" s="22" t="inlineStr">
+        <is>
+          <t>Patrol Snag (both pools)</t>
+        </is>
+      </c>
+      <c r="C111" s="22" t="inlineStr">
+        <is>
+          <t>Arcanine (Shadow)</t>
+        </is>
+      </c>
+      <c r="D111" s="22" t="inlineStr">
+        <is>
+          <t>43-44</t>
+        </is>
+      </c>
+      <c r="E111" s="22" t="inlineStr">
+        <is>
+          <t>pool of 15</t>
+        </is>
+      </c>
+      <c r="F111" s="22" t="inlineStr">
+        <is>
+          <t>Snag from patrol trainers</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="22" t="inlineStr">
+        <is>
+          <t>Shin-Tokyo (Red Alert)</t>
+        </is>
+      </c>
+      <c r="B112" s="22" t="inlineStr">
+        <is>
+          <t>Patrol Snag (both pools)</t>
+        </is>
+      </c>
+      <c r="C112" s="22" t="inlineStr">
+        <is>
+          <t>Marowak (Shadow)</t>
+        </is>
+      </c>
+      <c r="D112" s="22" t="inlineStr">
+        <is>
+          <t>43-44</t>
+        </is>
+      </c>
+      <c r="E112" s="22" t="inlineStr">
+        <is>
+          <t>pool of 15</t>
+        </is>
+      </c>
+      <c r="F112" s="22" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="22" t="inlineStr">
+        <is>
+          <t>Shin-Tokyo (Red Alert)</t>
+        </is>
+      </c>
+      <c r="B113" s="22" t="inlineStr">
+        <is>
+          <t>Patrol Snag (both pools)</t>
+        </is>
+      </c>
+      <c r="C113" s="22" t="inlineStr">
+        <is>
+          <t>Manectric (Shadow)</t>
+        </is>
+      </c>
+      <c r="D113" s="22" t="inlineStr">
+        <is>
+          <t>43-44</t>
+        </is>
+      </c>
+      <c r="E113" s="22" t="inlineStr">
+        <is>
+          <t>pool of 15</t>
+        </is>
+      </c>
+      <c r="F113" s="22" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="22" t="inlineStr">
+        <is>
+          <t>Shin-Tokyo (Red Alert)</t>
+        </is>
+      </c>
+      <c r="B114" s="22" t="inlineStr">
+        <is>
+          <t>Patrol Snag (both pools)</t>
+        </is>
+      </c>
+      <c r="C114" s="22" t="inlineStr">
+        <is>
+          <t>Luxray (Shadow)</t>
+        </is>
+      </c>
+      <c r="D114" s="22" t="inlineStr">
+        <is>
+          <t>43-44</t>
+        </is>
+      </c>
+      <c r="E114" s="22" t="inlineStr">
+        <is>
+          <t>pool of 15</t>
+        </is>
+      </c>
+      <c r="F114" s="22" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="22" t="inlineStr">
+        <is>
+          <t>Shin-Tokyo (Red Alert)</t>
+        </is>
+      </c>
+      <c r="B115" s="22" t="inlineStr">
+        <is>
+          <t>Patrol Snag (both pools)</t>
+        </is>
+      </c>
+      <c r="C115" s="22" t="inlineStr">
+        <is>
+          <t>Flygon (Shadow)</t>
+        </is>
+      </c>
+      <c r="D115" s="22" t="inlineStr">
+        <is>
+          <t>43-44</t>
+        </is>
+      </c>
+      <c r="E115" s="22" t="inlineStr">
+        <is>
+          <t>pool of 15</t>
+        </is>
+      </c>
+      <c r="F115" s="22" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="22" t="inlineStr">
+        <is>
+          <t>Shin-Tokyo (Red Alert)</t>
+        </is>
+      </c>
+      <c r="B116" s="22" t="inlineStr">
+        <is>
+          <t>Patrol Snag (both pools)</t>
+        </is>
+      </c>
+      <c r="C116" s="22" t="inlineStr">
+        <is>
+          <t>Venusaur (Shadow)</t>
+        </is>
+      </c>
+      <c r="D116" s="22" t="inlineStr">
+        <is>
+          <t>43-44</t>
+        </is>
+      </c>
+      <c r="E116" s="22" t="inlineStr">
+        <is>
+          <t>pool of 15</t>
+        </is>
+      </c>
+      <c r="F116" s="22" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="22" t="inlineStr">
+        <is>
+          <t>Shin-Tokyo Jail</t>
+        </is>
+      </c>
+      <c r="B117" s="22" t="inlineStr">
+        <is>
+          <t>Trainer Snag (JUZO squad)</t>
+        </is>
+      </c>
+      <c r="C117" s="22" t="inlineStr">
+        <is>
+          <t>Marowak (Shadow)</t>
+        </is>
+      </c>
+      <c r="D117" s="22" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E117" s="22" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
+      </c>
+      <c r="F117" s="22" t="inlineStr">
+        <is>
+          <t>Replaced Bronzong</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="22" t="inlineStr">
+        <is>
+          <t>Shin-Tokyo Jail</t>
+        </is>
+      </c>
+      <c r="B118" s="22" t="inlineStr">
+        <is>
+          <t>Trainer Snag (SAYA squad)</t>
+        </is>
+      </c>
+      <c r="C118" s="22" t="inlineStr">
+        <is>
+          <t>Luxray (Shadow)</t>
+        </is>
+      </c>
+      <c r="D118" s="22" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="E118" s="22" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
+      </c>
+      <c r="F118" s="22" t="inlineStr">
+        <is>
+          <t>Replaced Magnezone</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="22" t="inlineStr">
+        <is>
+          <t>Shin-Tokyo Dockhouse (post-game)</t>
+        </is>
+      </c>
+      <c r="B119" s="22" t="inlineStr">
+        <is>
+          <t>Trainer Reward</t>
+        </is>
+      </c>
+      <c r="C119" s="22" t="inlineStr">
+        <is>
+          <t>Mewtwo (Armored)</t>
+        </is>
+      </c>
+      <c r="D119" s="22" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="E119" s="22" t="inlineStr">
+        <is>
+          <t>one-time</t>
+        </is>
+      </c>
+      <c r="F119" s="22" t="inlineStr">
+        <is>
+          <t>Beat Draco after the post-game call; won, not caught</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F101"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3424,7 +3974,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3553,6 +4103,416 @@
         <v>82</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Celebi Island</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Route 129</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Route 130</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Shin-Tokyo (Red Alert)</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Shin-Tokyo Jail</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Shin-Tokyo Dockhouse (post-game)</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="B1" s="21" t="inlineStr">
+        <is>
+          <t>Custom Art By</t>
+        </is>
+      </c>
+      <c r="C1" s="21" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D1" s="21" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="22" t="inlineStr">
+        <is>
+          <t>Arceus</t>
+        </is>
+      </c>
+      <c r="B2" s="22" t="inlineStr">
+        <is>
+          <t>pogokitten</t>
+        </is>
+      </c>
+      <c r="C2" s="22" t="inlineStr">
+        <is>
+          <t>Art imported, no encounter</t>
+        </is>
+      </c>
+      <c r="D2" s="22" t="inlineStr">
+        <is>
+          <t>Battle sprite registered; not placed anywhere</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="22" t="inlineStr">
+        <is>
+          <t>Cresselia</t>
+        </is>
+      </c>
+      <c r="B3" s="22" t="inlineStr">
+        <is>
+          <t>pogokitten</t>
+        </is>
+      </c>
+      <c r="C3" s="22" t="inlineStr">
+        <is>
+          <t>Art imported, no encounter</t>
+        </is>
+      </c>
+      <c r="D3" s="22" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="22" t="inlineStr">
+        <is>
+          <t>Giratina</t>
+        </is>
+      </c>
+      <c r="B4" s="22" t="inlineStr">
+        <is>
+          <t>pogokitten</t>
+        </is>
+      </c>
+      <c r="C4" s="22" t="inlineStr">
+        <is>
+          <t>Art imported, no encounter</t>
+        </is>
+      </c>
+      <c r="D4" s="22" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="22" t="inlineStr">
+        <is>
+          <t>Suicune</t>
+        </is>
+      </c>
+      <c r="B5" s="22" t="inlineStr">
+        <is>
+          <t>pogokitten</t>
+        </is>
+      </c>
+      <c r="C5" s="22" t="inlineStr">
+        <is>
+          <t>Art imported, no encounter</t>
+        </is>
+      </c>
+      <c r="D5" s="22" t="inlineStr">
+        <is>
+          <t>Northwind Cavern Suicune is a NORMAL legendary, not Shadow</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="22" t="inlineStr">
+        <is>
+          <t>Typhlosion</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>pogokitten</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>Art imported, no encounter</t>
+        </is>
+      </c>
+      <c r="D6" s="22" t="inlineStr">
+        <is>
+          <t>StarSummit boss uses normal Typhlosion</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="22" t="inlineStr">
+        <is>
+          <t>Camerupt</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>pogokitten</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="inlineStr">
+        <is>
+          <t>Art imported, no encounter</t>
+        </is>
+      </c>
+      <c r="D7" s="22" t="inlineStr">
+        <is>
+          <t>From earlier waves</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="22" t="inlineStr">
+        <is>
+          <t>Charizard</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>pogokitten</t>
+        </is>
+      </c>
+      <c r="C8" s="22" t="inlineStr">
+        <is>
+          <t>Art imported, no encounter</t>
+        </is>
+      </c>
+      <c r="D8" s="22" t="inlineStr">
+        <is>
+          <t>Edwards dropped Shadow Charizard from his team</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="22" t="inlineStr">
+        <is>
+          <t>Charmeleon</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
+        <is>
+          <t>pogokitten</t>
+        </is>
+      </c>
+      <c r="C9" s="22" t="inlineStr">
+        <is>
+          <t>Art imported, no encounter</t>
+        </is>
+      </c>
+      <c r="D9" s="22" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="22" t="inlineStr">
+        <is>
+          <t>Chimchar</t>
+        </is>
+      </c>
+      <c r="B10" s="22" t="inlineStr">
+        <is>
+          <t>pogokitten</t>
+        </is>
+      </c>
+      <c r="C10" s="22" t="inlineStr">
+        <is>
+          <t>Art imported, no encounter</t>
+        </is>
+      </c>
+      <c r="D10" s="22" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="22" t="inlineStr">
+        <is>
+          <t>Dragonite</t>
+        </is>
+      </c>
+      <c r="B11" s="22" t="inlineStr">
+        <is>
+          <t>WeeGeeDude</t>
+        </is>
+      </c>
+      <c r="C11" s="22" t="inlineStr">
+        <is>
+          <t>Art imported, no encounter</t>
+        </is>
+      </c>
+      <c r="D11" s="22" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="22" t="inlineStr">
+        <is>
+          <t>Gallade</t>
+        </is>
+      </c>
+      <c r="B12" s="22" t="inlineStr">
+        <is>
+          <t>pogokitten</t>
+        </is>
+      </c>
+      <c r="C12" s="22" t="inlineStr">
+        <is>
+          <t>Art imported, no encounter</t>
+        </is>
+      </c>
+      <c r="D12" s="22" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="22" t="inlineStr">
+        <is>
+          <t>Gardevoir</t>
+        </is>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>pogokitten</t>
+        </is>
+      </c>
+      <c r="C13" s="22" t="inlineStr">
+        <is>
+          <t>Art imported, no encounter</t>
+        </is>
+      </c>
+      <c r="D13" s="22" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="22" t="inlineStr">
+        <is>
+          <t>Lugia</t>
+        </is>
+      </c>
+      <c r="B14" s="22" t="inlineStr">
+        <is>
+          <t>biadoxaf (sheet) / pogokitten</t>
+        </is>
+      </c>
+      <c r="C14" s="22" t="inlineStr">
+        <is>
+          <t>Art imported, no encounter</t>
+        </is>
+      </c>
+      <c r="D14" s="22" t="inlineStr">
+        <is>
+          <t>Endgame Rayquaza took the release slot</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="22" t="inlineStr">
+        <is>
+          <t>Pikachu</t>
+        </is>
+      </c>
+      <c r="B15" s="22" t="inlineStr">
+        <is>
+          <t>pogokitten</t>
+        </is>
+      </c>
+      <c r="C15" s="22" t="inlineStr">
+        <is>
+          <t>Art imported, no encounter</t>
+        </is>
+      </c>
+      <c r="D15" s="22" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="22" t="inlineStr">
+        <is>
+          <t>Turtwig</t>
+        </is>
+      </c>
+      <c r="B16" s="22" t="inlineStr">
+        <is>
+          <t>pogokitten</t>
+        </is>
+      </c>
+      <c r="C16" s="22" t="inlineStr">
+        <is>
+          <t>Art imported, no encounter</t>
+        </is>
+      </c>
+      <c r="D16" s="22" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>These species have finished Shadow battle art in graphics/pokemon_shadow/ but no obtainable encounter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Placing one in a wild table, snag team, or patrol pool makes it live; then APPEND it to the Shadow Log table (end only).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>